<commit_message>
fix: generating output with >16 channels
</commit_message>
<xml_diff>
--- a/templates/Yokogawa Hardware Conf.xlsx
+++ b/templates/Yokogawa Hardware Conf.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Working\Others\Python\Cloud App Projects\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Working\Others\Python\Cloud App Projects\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C11B95AE-9205-46A6-A1EA-328E33E81794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2EF2924-A642-4C0C-B791-A70CCA863788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Hardware Conf" sheetId="1" r:id="rId1"/>
     <sheet name="FIO" sheetId="3" r:id="rId2"/>
     <sheet name="Design Input Review" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="36">
   <si>
     <t>ESD</t>
   </si>
@@ -161,12 +162,30 @@
 If Individual Barrier - fall back to AI type wise segreation 
 If it is Barrier Board - then assign IOs in Separate Module</t>
   </si>
+  <si>
+    <t>Wired Spares %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IO Redundancy </t>
+  </si>
+  <si>
+    <t xml:space="preserve">IS/Non-IS Type </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Controller Model </t>
+  </si>
+  <si>
+    <t>Explosion Protection</t>
+  </si>
+  <si>
+    <t>Temperature Rating</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,6 +220,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF333333"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -238,7 +269,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -265,6 +296,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -984,4 +1017,87 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{958A5FC6-AD6B-4168-A87F-23D367259FC5}">
+  <dimension ref="C2:I7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:9" ht="20.399999999999999" x14ac:dyDescent="0.45">
+      <c r="C2" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+    </row>
+    <row r="3" spans="3:9" ht="20.399999999999999" x14ac:dyDescent="0.45">
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+    </row>
+    <row r="4" spans="3:9" ht="20.399999999999999" x14ac:dyDescent="0.45">
+      <c r="C4" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+    </row>
+    <row r="5" spans="3:9" ht="20.399999999999999" x14ac:dyDescent="0.45">
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+    </row>
+    <row r="6" spans="3:9" ht="20.399999999999999" x14ac:dyDescent="0.45">
+      <c r="C6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+    </row>
+    <row r="7" spans="3:9" ht="20.399999999999999" x14ac:dyDescent="0.45">
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
update: Design Input Review updated
</commit_message>
<xml_diff>
--- a/templates/Yokogawa Hardware Conf.xlsx
+++ b/templates/Yokogawa Hardware Conf.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Working\Others\Python\Cloud App Projects\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2EF2924-A642-4C0C-B791-A70CCA863788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97410CFF-900A-47DE-A64C-499715BB8F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="492" yWindow="1884" windowWidth="17280" windowHeight="8880" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hardware Conf" sheetId="1" r:id="rId1"/>
     <sheet name="FIO" sheetId="3" r:id="rId2"/>
     <sheet name="Design Input Review" sheetId="2" r:id="rId3"/>
     <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
+    <sheet name="Module Calculation" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -879,7 +880,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42EA331C-F9A1-4A1F-BFF3-07C529DB8C30}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="24.88671875" style="3" customWidth="1"/>
@@ -887,7 +888,7 @@
     <col min="4" max="4" width="16.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>24</v>
       </c>
@@ -901,7 +902,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -911,7 +912,7 @@
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -923,7 +924,7 @@
       </c>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -934,8 +935,30 @@
         <v>21</v>
       </c>
       <c r="D4" s="4"/>
-    </row>
-    <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="H4">
+        <v>148</v>
+      </c>
+      <c r="I4">
+        <v>16</v>
+      </c>
+      <c r="J4">
+        <f>H4/I4</f>
+        <v>9.25</v>
+      </c>
+      <c r="K4">
+        <f>ROUNDUP(J4, 0)</f>
+        <v>10</v>
+      </c>
+      <c r="L4">
+        <f>I4*K4</f>
+        <v>160</v>
+      </c>
+      <c r="M4">
+        <f>L4-H4</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -946,8 +969,38 @@
         <v>27</v>
       </c>
       <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="H5">
+        <v>324</v>
+      </c>
+      <c r="I5">
+        <v>16</v>
+      </c>
+      <c r="J5">
+        <f t="shared" ref="J5:J6" si="0">H5/I5</f>
+        <v>20.25</v>
+      </c>
+      <c r="K5">
+        <f t="shared" ref="K5:K6" si="1">ROUNDUP(J5, 0)</f>
+        <v>21</v>
+      </c>
+      <c r="L5">
+        <f t="shared" ref="L5:L6" si="2">I5*K5</f>
+        <v>336</v>
+      </c>
+      <c r="M5">
+        <f t="shared" ref="M5:M6" si="3">L5-H5</f>
+        <v>12</v>
+      </c>
+      <c r="O5">
+        <f>555*0.2+555</f>
+        <v>666</v>
+      </c>
+      <c r="P5">
+        <f>O5/16</f>
+        <v>41.625</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -958,8 +1011,30 @@
         <v>28</v>
       </c>
       <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="H6">
+        <v>194</v>
+      </c>
+      <c r="I6">
+        <v>16</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="0"/>
+        <v>12.125</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+      <c r="L6">
+        <f t="shared" si="2"/>
+        <v>208</v>
+      </c>
+      <c r="M6">
+        <f t="shared" si="3"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -968,8 +1043,20 @@
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:4" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="K7">
+        <f>SUM(K4:K6)</f>
+        <v>44</v>
+      </c>
+      <c r="L7">
+        <f t="shared" ref="L7:M7" si="4">SUM(L4:L6)</f>
+        <v>704</v>
+      </c>
+      <c r="M7">
+        <f t="shared" si="4"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="5"/>
       <c r="C8" s="8" t="s">
@@ -977,37 +1064,37 @@
       </c>
       <c r="D8" s="4"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" s="5"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="5"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" s="5"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="5"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="5"/>
       <c r="C14" s="4"/>
@@ -1100,4 +1187,188 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E954E18D-B3BC-4CEE-BA2B-E89B3B056095}">
+  <dimension ref="A2:K13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>93</v>
+      </c>
+      <c r="B2">
+        <v>30</v>
+      </c>
+      <c r="C2">
+        <v>148</v>
+      </c>
+      <c r="D2">
+        <v>16</v>
+      </c>
+      <c r="E2">
+        <f>C2/D2</f>
+        <v>9.25</v>
+      </c>
+      <c r="F2">
+        <f>ROUNDUP(E2, 0)</f>
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <f>D2*F2</f>
+        <v>160</v>
+      </c>
+      <c r="H2">
+        <f>G2-C2</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>110</v>
+      </c>
+      <c r="B3">
+        <v>160</v>
+      </c>
+      <c r="C3">
+        <v>324</v>
+      </c>
+      <c r="D3">
+        <v>16</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E4" si="0">C3/D3</f>
+        <v>20.25</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F4" si="1">ROUNDUP(E3, 0)</f>
+        <v>21</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G4" si="2">D3*F3</f>
+        <v>336</v>
+      </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H4" si="3">G3-C3</f>
+        <v>12</v>
+      </c>
+      <c r="J3">
+        <f>555*0.2+555</f>
+        <v>666</v>
+      </c>
+      <c r="K3">
+        <f>J3/16</f>
+        <v>41.625</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>45</v>
+      </c>
+      <c r="B4">
+        <v>117</v>
+      </c>
+      <c r="C4">
+        <v>194</v>
+      </c>
+      <c r="D4">
+        <v>16</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>12.125</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="1"/>
+        <v>13</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="2"/>
+        <v>208</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="3"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C5">
+        <f>SUM(C2:C4)</f>
+        <v>666</v>
+      </c>
+      <c r="F5">
+        <f>SUM(F2:F4)</f>
+        <v>44</v>
+      </c>
+      <c r="G5">
+        <f t="shared" ref="G5:H5" si="4">SUM(G2:G4)</f>
+        <v>704</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="4"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C6">
+        <f>C5/16</f>
+        <v>41.625</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="D8">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C9">
+        <v>120</v>
+      </c>
+      <c r="D9">
+        <v>22.5</v>
+      </c>
+      <c r="E9">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C10">
+        <v>100</v>
+      </c>
+      <c r="D10">
+        <v>19.5</v>
+      </c>
+      <c r="E10">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C11">
+        <v>100</v>
+      </c>
+      <c r="D11">
+        <v>19.399999999999999</v>
+      </c>
+      <c r="E11">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C12">
+        <v>80</v>
+      </c>
+      <c r="D12">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C13">
+        <f>SUM(C9:C12)</f>
+        <v>400</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>